<commit_message>
feat: finalize Preview website inquiry to quote snapshots and templates
</commit_message>
<xml_diff>
--- a/src/assets/quote-templates/ROMIKU_报价单_模板.xlsx
+++ b/src/assets/quote-templates/ROMIKU_报价单_模板.xlsx
@@ -4,13 +4,13 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView windowHeight="15480"/>
+    <workbookView windowHeight="15280"/>
   </bookViews>
   <sheets>
     <sheet name="ROMIKU PI" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'ROMIKU PI'!$A$1:$H$11</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'ROMIKU PI'!$A$1:$H$12</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
   <si>
     <t xml:space="preserve">                                      REQUEST FOR A QUOTE</t>
   </si>
@@ -43,6 +43,12 @@
 2026.9.23</t>
   </si>
   <si>
+    <t>供应商信息/SUPPLIER INFORMATION</t>
+  </si>
+  <si>
+    <t>客户信息/CUSTOMER INFORMATION</t>
+  </si>
+  <si>
     <t>COMPANY /NAME
 公司名称</t>
   </si>
@@ -54,7 +60,7 @@
 地址</t>
   </si>
   <si>
-    <t>72790, 3rd Street, Unit 4, 2nd Floor, Gate 153,Global Digital Trade Center Yiwu,China
+    <t>72790, 3rd Street, Unit 4, 2nd Floor, Gate 153,Global Digital Trade Center Yiwu
 义乌市国际商贸城六区152号门2楼4单元3街72790 </t>
   </si>
   <si>
@@ -560,6 +566,56 @@
     </border>
     <border>
       <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right/>
       <top/>
       <bottom style="thin">
@@ -572,59 +628,7 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
       <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
@@ -903,18 +907,27 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="49" applyFont="1"/>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="49" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -922,16 +935,19 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="7" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -940,37 +956,28 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="8" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="3" fillId="3" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="3" fillId="3" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -979,7 +986,7 @@
     <xf numFmtId="176" fontId="5" fillId="0" borderId="3" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="6" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="5" fillId="0" borderId="2" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="49" applyFont="1"/>
@@ -1479,7 +1486,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.8" outlineLevelCol="7"/>
   <cols>
     <col min="2" max="2" width="29.7788461538462" customWidth="1"/>
@@ -1511,225 +1518,256 @@
         <v>3</v>
       </c>
       <c r="B2" s="6"/>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
       <c r="F2" s="8"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="10"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
     </row>
     <row r="3" ht="55" customHeight="1" spans="1:8">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="11"/>
-      <c r="C3" s="12" t="s">
+      <c r="B3" s="9"/>
+      <c r="C3" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="12" t="s">
+        <v>5</v>
+      </c>
       <c r="F3" s="13"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="15"/>
-    </row>
-    <row r="4" ht="55" customHeight="1" spans="1:8">
-      <c r="A4" s="11" t="s">
+      <c r="G3" s="13"/>
+      <c r="H3" s="14"/>
+    </row>
+    <row r="4" ht="72" customHeight="1" spans="1:8">
+      <c r="A4" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="11"/>
-      <c r="C4" s="37" t="s">
+      <c r="B4" s="15"/>
+      <c r="C4" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="12" t="s">
+        <v>7</v>
+      </c>
       <c r="F4" s="13"/>
-      <c r="G4" s="14"/>
-      <c r="H4" s="15"/>
+      <c r="G4" s="13"/>
+      <c r="H4" s="14"/>
     </row>
     <row r="5" ht="55" customHeight="1" spans="1:8">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="11"/>
-      <c r="C5" s="16" t="s">
+      <c r="B5" s="15"/>
+      <c r="C5" s="38" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="18"/>
-      <c r="H5" s="19"/>
+      <c r="E5" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="14"/>
     </row>
     <row r="6" ht="55" customHeight="1" spans="1:8">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="11"/>
-      <c r="C6" s="16" t="s">
+      <c r="B6" s="15"/>
+      <c r="C6" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="19"/>
-    </row>
-    <row r="7" ht="47" customHeight="1" spans="1:8">
-      <c r="A7" s="20" t="s">
+      <c r="D6" s="19"/>
+      <c r="E6" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="14"/>
+    </row>
+    <row r="7" ht="55" customHeight="1" spans="1:8">
+      <c r="A7" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="15"/>
+      <c r="C7" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="D7" s="19"/>
+      <c r="E7" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="14"/>
+    </row>
+    <row r="8" ht="47" customHeight="1" spans="1:8">
+      <c r="A8" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="B8" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="20" t="s">
+      <c r="C8" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="20" t="s">
+      <c r="D8" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="21" t="s">
+      <c r="E8" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="H7" s="21" t="s">
+      <c r="F8" s="21" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="8" ht="100" customHeight="1" spans="1:8">
-      <c r="A8" s="22">
+      <c r="G8" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" s="22" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" ht="100" customHeight="1" spans="1:8">
+      <c r="A9" s="23">
         <v>1</v>
       </c>
-      <c r="B8" s="22"/>
-      <c r="C8" s="22"/>
-      <c r="D8" s="23"/>
-      <c r="E8" s="22"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="22"/>
-      <c r="H8" s="22"/>
-    </row>
-    <row r="9" ht="100" customHeight="1" spans="1:8">
-      <c r="A9" s="22">
+      <c r="B9" s="23"/>
+      <c r="C9" s="23"/>
+      <c r="D9" s="24"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+    </row>
+    <row r="10" ht="100" customHeight="1" spans="1:8">
+      <c r="A10" s="23">
         <v>2</v>
       </c>
-      <c r="B9" s="22"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="26"/>
-      <c r="H9" s="26"/>
-    </row>
-    <row r="10" ht="100" customHeight="1" spans="1:8">
-      <c r="A10" s="22">
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="26"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="27"/>
+    </row>
+    <row r="11" ht="100" customHeight="1" spans="1:8">
+      <c r="A11" s="23">
         <v>3</v>
       </c>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="26"/>
-      <c r="H10" s="26"/>
-    </row>
-    <row r="11" ht="100" customHeight="1" spans="1:8">
-      <c r="A11" s="22">
-        <v>4</v>
-      </c>
-      <c r="B11" s="22"/>
-      <c r="C11" s="22"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="24"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
+      <c r="D11" s="24"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="26"/>
       <c r="G11" s="27"/>
       <c r="H11" s="27"/>
     </row>
-    <row r="12" s="1" customFormat="1" ht="24" customHeight="1" spans="1:8">
-      <c r="A12" s="28"/>
-      <c r="B12" s="29"/>
-      <c r="C12" s="29"/>
-      <c r="D12" s="29"/>
-      <c r="E12" s="29"/>
-      <c r="F12" s="29"/>
-      <c r="G12" s="30"/>
-      <c r="H12" s="30"/>
-    </row>
-    <row r="13" ht="40" customHeight="1" spans="1:8">
-      <c r="B13" s="31"/>
-      <c r="C13" s="31"/>
-      <c r="D13" s="31"/>
-      <c r="E13" s="31"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="33"/>
-      <c r="H13" s="33"/>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="C14" s="34"/>
-      <c r="D14" s="34"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="34"/>
-      <c r="G14" s="35"/>
-      <c r="H14" s="35"/>
+    <row r="12" ht="100" customHeight="1" spans="1:8">
+      <c r="A12" s="23">
+        <v>4</v>
+      </c>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="25"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="28"/>
+    </row>
+    <row r="13" s="1" customFormat="1" ht="24" customHeight="1" spans="1:8">
+      <c r="A13" s="29"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="30"/>
+      <c r="D13" s="30"/>
+      <c r="E13" s="30"/>
+      <c r="F13" s="30"/>
+      <c r="G13" s="31"/>
+      <c r="H13" s="31"/>
+    </row>
+    <row r="14" ht="40" customHeight="1" spans="1:8">
+      <c r="B14" s="32"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="32"/>
+      <c r="E14" s="32"/>
+      <c r="F14" s="33"/>
+      <c r="G14" s="34"/>
+      <c r="H14" s="34"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="B15" s="32"/>
-      <c r="C15" s="32"/>
-      <c r="D15" s="32"/>
-      <c r="E15" s="32"/>
-      <c r="F15" s="32"/>
-      <c r="G15" s="33"/>
-      <c r="H15" s="33"/>
+      <c r="C15" s="35"/>
+      <c r="D15" s="35"/>
+      <c r="E15" s="35"/>
+      <c r="F15" s="35"/>
+      <c r="G15" s="36"/>
+      <c r="H15" s="36"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="B16" s="32"/>
-      <c r="C16" s="32"/>
-      <c r="D16" s="32"/>
-      <c r="E16" s="32"/>
-      <c r="F16" s="32"/>
-      <c r="G16" s="33"/>
-      <c r="H16" s="33"/>
+      <c r="B16" s="33"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="34"/>
+      <c r="H16" s="34"/>
     </row>
     <row r="17" spans="2:8">
-      <c r="B17" s="32"/>
-      <c r="C17" s="32"/>
-      <c r="D17" s="32"/>
-      <c r="E17" s="32"/>
-      <c r="F17" s="32"/>
-      <c r="G17" s="33"/>
-      <c r="H17" s="33"/>
+      <c r="B17" s="33"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="33"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="33"/>
+      <c r="G17" s="34"/>
+      <c r="H17" s="34"/>
     </row>
     <row r="18" spans="2:8">
-      <c r="B18" s="32"/>
-      <c r="C18" s="32"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="33"/>
-      <c r="H18" s="33"/>
-    </row>
-    <row r="39" spans="3:3">
-      <c r="C39" s="36"/>
+      <c r="B18" s="33"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="33"/>
+      <c r="E18" s="33"/>
+      <c r="F18" s="33"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="34"/>
+    </row>
+    <row r="19" spans="2:8">
+      <c r="B19" s="33"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="34"/>
+    </row>
+    <row r="40" spans="3:3">
+      <c r="C40" s="37"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="19">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="C2:H2"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="E2:H2"/>
     <mergeCell ref="A3:B3"/>
-    <mergeCell ref="C3:H3"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="C4:H4"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="F4:H4"/>
     <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="F5:H5"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="C6:H6"/>
-    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="F7:H7"/>
+    <mergeCell ref="B13:H13"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.12" footer="0.12"/>

</xml_diff>